<commit_message>
Añadir prototipo del parser del excel de horarios, creando un archivo para ello
</commit_message>
<xml_diff>
--- a/app_horarios/datos/excel/export-15-04.xlsx
+++ b/app_horarios/datos/excel/export-15-04.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F0A45E-9DC8-43E0-8805-C456A9AFB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="11" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="asignaturas" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,20 @@
     <sheet name="tfg" sheetId="18" r:id="rId18"/>
     <sheet name="usuarios" sheetId="19" r:id="rId19"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -751,7 +764,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -809,7 +822,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>

<commit_message>
Hacer cambios para poder modificar el estado, que no se enviaba al back. Y hacer que cuando se modifiquen fechas o recursos del aula obligue a buscar de nuevo un aula
</commit_message>
<xml_diff>
--- a/app_horarios/datos/excel/export-15-04.xlsx
+++ b/app_horarios/datos/excel/export-15-04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Desktop\Ingeniería informática\4º Trabajo de Fin de Grado\Trabajo-Fin-de-Grado-2025-2026\app_horarios\datos\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86D8BE3B-B62A-4F90-AC16-170140AFF7EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52115464-5F14-462F-868F-4460992DB328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="asignaturas" sheetId="1" r:id="rId1"/>
@@ -8727,7 +8727,7 @@
         <v>6392</v>
       </c>
       <c r="E2">
-        <v>25</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Añadir el traceback para ver dónde falla y añadir el Aula 0 en base de datos
</commit_message>
<xml_diff>
--- a/app_horarios/datos/excel/export-15-04.xlsx
+++ b/app_horarios/datos/excel/export-15-04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Desktop\Ingeniería informática\4º Trabajo de Fin de Grado\Trabajo-Fin-de-Grado-2025-2026\app_horarios\datos\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E5D0545-00F3-4165-92C4-376C6897CCA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06F8DCF0-5CDF-4DBA-AC33-6495C1219F55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="asignaturas" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1864" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1866" uniqueCount="582">
   <si>
     <t>IDASIGNATURA</t>
   </si>
@@ -1797,6 +1797,9 @@
   </si>
   <si>
     <t>Lab 46-A1</t>
+  </si>
+  <si>
+    <t>Aula 0</t>
   </si>
 </sst>
 </file>
@@ -2262,6 +2265,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="44.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -15628,7 +15632,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="25.6640625" bestFit="1" customWidth="1"/>
@@ -17237,6 +17241,17 @@
         <v>267</v>
       </c>
       <c r="O60" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>581</v>
+      </c>
+      <c r="O61" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Aplicar modificación de cmabios teórcios, hacer que haga una reserva por cada día lectivo correspondiente, corregir errores para el funcionamiento de la creación de las reservas periódicas y hacer el identificador de las reservas autoincremental en base de datos
</commit_message>
<xml_diff>
--- a/app_horarios/datos/excel/export-15-04.xlsx
+++ b/app_horarios/datos/excel/export-15-04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Desktop\Ingeniería informática\4º Trabajo de Fin de Grado\Trabajo-Fin-de-Grado-2025-2026\app_horarios\datos\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06F8DCF0-5CDF-4DBA-AC33-6495C1219F55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0932203-CB09-4436-8A1E-E503933AFB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="asignaturas" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1866" uniqueCount="582">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1836" uniqueCount="567">
   <si>
     <t>IDASIGNATURA</t>
   </si>
@@ -398,9 +398,6 @@
     <t>HORA_FIN</t>
   </si>
   <si>
-    <t>R0001</t>
-  </si>
-  <si>
     <t>P</t>
   </si>
   <si>
@@ -410,18 +407,12 @@
     <t>17:43:00</t>
   </si>
   <si>
-    <t>R0002</t>
-  </si>
-  <si>
     <t>18:00:00</t>
   </si>
   <si>
     <t>19:00:00</t>
   </si>
   <si>
-    <t>R0003</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
@@ -431,9 +422,6 @@
     <t>12:00:00</t>
   </si>
   <si>
-    <t>R0004</t>
-  </si>
-  <si>
     <t>R</t>
   </si>
   <si>
@@ -443,61 +431,28 @@
     <t>15:00:00</t>
   </si>
   <si>
-    <t>R0005</t>
-  </si>
-  <si>
     <t>16:00:00</t>
   </si>
   <si>
-    <t>R0006</t>
-  </si>
-  <si>
     <t>11:00:00</t>
   </si>
   <si>
-    <t>R0007</t>
-  </si>
-  <si>
-    <t>R0008</t>
-  </si>
-  <si>
-    <t>R0009</t>
-  </si>
-  <si>
-    <t>R0010</t>
-  </si>
-  <si>
     <t>16:30:00</t>
   </si>
   <si>
     <t>18:30:00</t>
   </si>
   <si>
-    <t>R0011</t>
-  </si>
-  <si>
-    <t>R0012</t>
-  </si>
-  <si>
-    <t>R0013</t>
-  </si>
-  <si>
     <t>11:30:00</t>
   </si>
   <si>
     <t>12:30:00</t>
   </si>
   <si>
-    <t>R0014</t>
-  </si>
-  <si>
     <t>17:28:00</t>
   </si>
   <si>
     <t>18:29:00</t>
-  </si>
-  <si>
-    <t>R0015</t>
   </si>
   <si>
     <t>17:00:00</t>
@@ -2302,7 +2257,7 @@
         <v>8797</v>
       </c>
       <c r="B2" t="s">
-        <v>270</v>
+        <v>255</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -2365,7 +2320,7 @@
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -2392,10 +2347,10 @@
         <v>8800</v>
       </c>
       <c r="B5" t="s">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="C5" t="s">
-        <v>273</v>
+        <v>258</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -2422,10 +2377,10 @@
         <v>8796</v>
       </c>
       <c r="B6" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="C6" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -2452,10 +2407,10 @@
         <v>8801</v>
       </c>
       <c r="B7" t="s">
-        <v>276</v>
+        <v>261</v>
       </c>
       <c r="C7" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -2482,10 +2437,10 @@
         <v>8802</v>
       </c>
       <c r="B8" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="C8" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -2512,10 +2467,10 @@
         <v>8803</v>
       </c>
       <c r="B9" t="s">
-        <v>280</v>
+        <v>265</v>
       </c>
       <c r="C9" t="s">
-        <v>281</v>
+        <v>266</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -2542,10 +2497,10 @@
         <v>8804</v>
       </c>
       <c r="B10" t="s">
-        <v>282</v>
+        <v>267</v>
       </c>
       <c r="C10" t="s">
-        <v>283</v>
+        <v>268</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -2572,10 +2527,10 @@
         <v>8805</v>
       </c>
       <c r="B11" t="s">
-        <v>284</v>
+        <v>269</v>
       </c>
       <c r="C11" t="s">
-        <v>285</v>
+        <v>270</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -2602,10 +2557,10 @@
         <v>8806</v>
       </c>
       <c r="B12" t="s">
-        <v>286</v>
+        <v>271</v>
       </c>
       <c r="C12" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
       <c r="D12">
         <v>2</v>
@@ -2632,10 +2587,10 @@
         <v>8807</v>
       </c>
       <c r="B13" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="C13" t="s">
-        <v>289</v>
+        <v>274</v>
       </c>
       <c r="D13">
         <v>2</v>
@@ -2662,10 +2617,10 @@
         <v>8808</v>
       </c>
       <c r="B14" t="s">
-        <v>290</v>
+        <v>275</v>
       </c>
       <c r="C14" t="s">
-        <v>291</v>
+        <v>276</v>
       </c>
       <c r="D14">
         <v>2</v>
@@ -2692,10 +2647,10 @@
         <v>8809</v>
       </c>
       <c r="B15" t="s">
-        <v>292</v>
+        <v>277</v>
       </c>
       <c r="C15" t="s">
-        <v>293</v>
+        <v>278</v>
       </c>
       <c r="D15">
         <v>2</v>
@@ -2722,10 +2677,10 @@
         <v>8810</v>
       </c>
       <c r="B16" t="s">
-        <v>294</v>
+        <v>279</v>
       </c>
       <c r="C16" t="s">
-        <v>295</v>
+        <v>280</v>
       </c>
       <c r="D16">
         <v>2</v>
@@ -2752,10 +2707,10 @@
         <v>8811</v>
       </c>
       <c r="B17" t="s">
-        <v>296</v>
+        <v>281</v>
       </c>
       <c r="C17" t="s">
-        <v>297</v>
+        <v>282</v>
       </c>
       <c r="D17">
         <v>2</v>
@@ -2782,10 +2737,10 @@
         <v>8812</v>
       </c>
       <c r="B18" t="s">
-        <v>298</v>
+        <v>283</v>
       </c>
       <c r="C18" t="s">
-        <v>299</v>
+        <v>284</v>
       </c>
       <c r="D18">
         <v>2</v>
@@ -2812,10 +2767,10 @@
         <v>8813</v>
       </c>
       <c r="B19" t="s">
-        <v>300</v>
+        <v>285</v>
       </c>
       <c r="C19" t="s">
-        <v>301</v>
+        <v>286</v>
       </c>
       <c r="D19">
         <v>2</v>
@@ -2842,10 +2797,10 @@
         <v>8814</v>
       </c>
       <c r="B20" t="s">
-        <v>302</v>
+        <v>287</v>
       </c>
       <c r="C20" t="s">
-        <v>303</v>
+        <v>288</v>
       </c>
       <c r="D20">
         <v>2</v>
@@ -2872,10 +2827,10 @@
         <v>8815</v>
       </c>
       <c r="B21" t="s">
-        <v>304</v>
+        <v>289</v>
       </c>
       <c r="C21" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
       <c r="D21">
         <v>2</v>
@@ -2902,10 +2857,10 @@
         <v>8816</v>
       </c>
       <c r="B22" t="s">
-        <v>306</v>
+        <v>291</v>
       </c>
       <c r="C22" t="s">
-        <v>307</v>
+        <v>292</v>
       </c>
       <c r="D22">
         <v>3</v>
@@ -2932,10 +2887,10 @@
         <v>8817</v>
       </c>
       <c r="B23" t="s">
-        <v>308</v>
+        <v>293</v>
       </c>
       <c r="C23" t="s">
-        <v>309</v>
+        <v>294</v>
       </c>
       <c r="D23">
         <v>3</v>
@@ -2962,10 +2917,10 @@
         <v>8818</v>
       </c>
       <c r="B24" t="s">
-        <v>310</v>
+        <v>295</v>
       </c>
       <c r="C24" t="s">
-        <v>311</v>
+        <v>296</v>
       </c>
       <c r="D24">
         <v>3</v>
@@ -2992,10 +2947,10 @@
         <v>8819</v>
       </c>
       <c r="B25" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="C25" t="s">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="D25">
         <v>3</v>
@@ -3022,10 +2977,10 @@
         <v>8820</v>
       </c>
       <c r="B26" t="s">
-        <v>314</v>
+        <v>299</v>
       </c>
       <c r="C26" t="s">
-        <v>315</v>
+        <v>300</v>
       </c>
       <c r="D26">
         <v>3</v>
@@ -3052,10 +3007,10 @@
         <v>8824</v>
       </c>
       <c r="B27" t="s">
-        <v>316</v>
+        <v>301</v>
       </c>
       <c r="C27" t="s">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="D27">
         <v>3</v>
@@ -3082,10 +3037,10 @@
         <v>8823</v>
       </c>
       <c r="B28" t="s">
-        <v>318</v>
+        <v>303</v>
       </c>
       <c r="C28" t="s">
-        <v>319</v>
+        <v>304</v>
       </c>
       <c r="D28">
         <v>3</v>
@@ -3112,10 +3067,10 @@
         <v>8825</v>
       </c>
       <c r="B29" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="C29" t="s">
-        <v>321</v>
+        <v>306</v>
       </c>
       <c r="D29">
         <v>3</v>
@@ -3142,10 +3097,10 @@
         <v>8821</v>
       </c>
       <c r="B30" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="C30" t="s">
-        <v>323</v>
+        <v>308</v>
       </c>
       <c r="D30">
         <v>3</v>
@@ -3172,10 +3127,10 @@
         <v>8822</v>
       </c>
       <c r="B31" t="s">
-        <v>324</v>
+        <v>309</v>
       </c>
       <c r="C31" t="s">
-        <v>325</v>
+        <v>310</v>
       </c>
       <c r="D31">
         <v>3</v>
@@ -3202,10 +3157,10 @@
         <v>8827</v>
       </c>
       <c r="B32" t="s">
-        <v>326</v>
+        <v>311</v>
       </c>
       <c r="C32" t="s">
-        <v>327</v>
+        <v>312</v>
       </c>
       <c r="D32">
         <v>4</v>
@@ -3221,7 +3176,7 @@
         <v>281</v>
       </c>
       <c r="H32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I32">
         <v>2</v>
@@ -3232,10 +3187,10 @@
         <v>8828</v>
       </c>
       <c r="B33" t="s">
-        <v>328</v>
+        <v>313</v>
       </c>
       <c r="C33" t="s">
-        <v>329</v>
+        <v>314</v>
       </c>
       <c r="D33">
         <v>4</v>
@@ -3251,7 +3206,7 @@
         <v>281</v>
       </c>
       <c r="H33" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I33">
         <v>2</v>
@@ -3262,10 +3217,10 @@
         <v>8829</v>
       </c>
       <c r="B34" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
       <c r="C34" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
       <c r="D34">
         <v>4</v>
@@ -3281,7 +3236,7 @@
         <v>281</v>
       </c>
       <c r="H34" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I34">
         <v>2</v>
@@ -3292,10 +3247,10 @@
         <v>8830</v>
       </c>
       <c r="B35" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
       <c r="C35" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
       <c r="D35">
         <v>4</v>
@@ -3311,7 +3266,7 @@
         <v>281</v>
       </c>
       <c r="H35" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I35">
         <v>2</v>
@@ -3322,10 +3277,10 @@
         <v>8831</v>
       </c>
       <c r="B36" t="s">
-        <v>334</v>
+        <v>319</v>
       </c>
       <c r="C36" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
       <c r="D36">
         <v>4</v>
@@ -3341,7 +3296,7 @@
         <v>281</v>
       </c>
       <c r="H36" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I36">
         <v>2</v>
@@ -3352,10 +3307,10 @@
         <v>8832</v>
       </c>
       <c r="B37" t="s">
-        <v>336</v>
+        <v>321</v>
       </c>
       <c r="C37" t="s">
-        <v>337</v>
+        <v>322</v>
       </c>
       <c r="D37">
         <v>4</v>
@@ -3371,7 +3326,7 @@
         <v>281</v>
       </c>
       <c r="H37" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I37">
         <v>2</v>
@@ -3382,10 +3337,10 @@
         <v>8833</v>
       </c>
       <c r="B38" t="s">
-        <v>338</v>
+        <v>323</v>
       </c>
       <c r="C38" t="s">
-        <v>339</v>
+        <v>324</v>
       </c>
       <c r="D38">
         <v>4</v>
@@ -3401,7 +3356,7 @@
         <v>281</v>
       </c>
       <c r="H38" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I38">
         <v>2</v>
@@ -3412,10 +3367,10 @@
         <v>8834</v>
       </c>
       <c r="B39" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
       <c r="C39" t="s">
-        <v>341</v>
+        <v>326</v>
       </c>
       <c r="D39">
         <v>4</v>
@@ -3431,7 +3386,7 @@
         <v>281</v>
       </c>
       <c r="H39" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I39">
         <v>2</v>
@@ -3442,10 +3397,10 @@
         <v>8835</v>
       </c>
       <c r="B40" t="s">
-        <v>342</v>
+        <v>327</v>
       </c>
       <c r="C40" t="s">
-        <v>343</v>
+        <v>328</v>
       </c>
       <c r="D40">
         <v>4</v>
@@ -3461,7 +3416,7 @@
         <v>281</v>
       </c>
       <c r="H40" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I40">
         <v>2</v>
@@ -3472,10 +3427,10 @@
         <v>8836</v>
       </c>
       <c r="B41" t="s">
-        <v>344</v>
+        <v>329</v>
       </c>
       <c r="C41" t="s">
-        <v>345</v>
+        <v>330</v>
       </c>
       <c r="D41">
         <v>4</v>
@@ -3491,7 +3446,7 @@
         <v>281</v>
       </c>
       <c r="H41" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I41">
         <v>2</v>
@@ -3502,10 +3457,10 @@
         <v>8837</v>
       </c>
       <c r="B42" t="s">
-        <v>346</v>
+        <v>331</v>
       </c>
       <c r="C42" t="s">
-        <v>347</v>
+        <v>332</v>
       </c>
       <c r="D42">
         <v>4</v>
@@ -3521,7 +3476,7 @@
         <v>281</v>
       </c>
       <c r="H42" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I42">
         <v>2</v>
@@ -3532,10 +3487,10 @@
         <v>8838</v>
       </c>
       <c r="B43" t="s">
-        <v>348</v>
+        <v>333</v>
       </c>
       <c r="C43" t="s">
-        <v>349</v>
+        <v>334</v>
       </c>
       <c r="D43">
         <v>4</v>
@@ -3551,7 +3506,7 @@
         <v>281</v>
       </c>
       <c r="H43" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I43">
         <v>2</v>
@@ -3562,10 +3517,10 @@
         <v>8842</v>
       </c>
       <c r="B44" t="s">
-        <v>350</v>
+        <v>335</v>
       </c>
       <c r="C44" t="s">
-        <v>351</v>
+        <v>336</v>
       </c>
       <c r="D44">
         <v>4</v>
@@ -3581,7 +3536,7 @@
         <v>281</v>
       </c>
       <c r="H44" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I44">
         <v>2</v>
@@ -3592,10 +3547,10 @@
         <v>8843</v>
       </c>
       <c r="B45" t="s">
-        <v>352</v>
+        <v>337</v>
       </c>
       <c r="C45" t="s">
-        <v>353</v>
+        <v>338</v>
       </c>
       <c r="D45">
         <v>4</v>
@@ -3611,7 +3566,7 @@
         <v>281</v>
       </c>
       <c r="H45" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I45">
         <v>2</v>
@@ -3622,7 +3577,7 @@
         <v>6392</v>
       </c>
       <c r="B46" t="s">
-        <v>354</v>
+        <v>339</v>
       </c>
       <c r="C46" t="s">
         <v>9</v>
@@ -3652,10 +3607,10 @@
         <v>6393</v>
       </c>
       <c r="B47" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="C47" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="D47">
         <v>1</v>
@@ -3682,10 +3637,10 @@
         <v>6394</v>
       </c>
       <c r="B48" t="s">
-        <v>355</v>
+        <v>340</v>
       </c>
       <c r="C48" t="s">
-        <v>356</v>
+        <v>341</v>
       </c>
       <c r="D48">
         <v>1</v>
@@ -3712,10 +3667,10 @@
         <v>6395</v>
       </c>
       <c r="B49" t="s">
-        <v>357</v>
+        <v>342</v>
       </c>
       <c r="C49" t="s">
-        <v>358</v>
+        <v>343</v>
       </c>
       <c r="D49">
         <v>1</v>
@@ -3772,10 +3727,10 @@
         <v>6397</v>
       </c>
       <c r="B51" t="s">
-        <v>359</v>
+        <v>344</v>
       </c>
       <c r="C51" t="s">
-        <v>360</v>
+        <v>345</v>
       </c>
       <c r="D51">
         <v>1</v>
@@ -3802,10 +3757,10 @@
         <v>6398</v>
       </c>
       <c r="B52" t="s">
-        <v>361</v>
+        <v>346</v>
       </c>
       <c r="C52" t="s">
-        <v>362</v>
+        <v>347</v>
       </c>
       <c r="D52">
         <v>1</v>
@@ -3832,10 +3787,10 @@
         <v>6399</v>
       </c>
       <c r="B53" t="s">
-        <v>363</v>
+        <v>348</v>
       </c>
       <c r="C53" t="s">
-        <v>364</v>
+        <v>349</v>
       </c>
       <c r="D53">
         <v>1</v>
@@ -3862,10 +3817,10 @@
         <v>6400</v>
       </c>
       <c r="B54" t="s">
-        <v>365</v>
+        <v>350</v>
       </c>
       <c r="C54" t="s">
-        <v>366</v>
+        <v>351</v>
       </c>
       <c r="D54">
         <v>1</v>
@@ -3892,10 +3847,10 @@
         <v>6401</v>
       </c>
       <c r="B55" t="s">
-        <v>367</v>
+        <v>352</v>
       </c>
       <c r="C55" t="s">
-        <v>368</v>
+        <v>353</v>
       </c>
       <c r="D55">
         <v>1</v>
@@ -3922,10 +3877,10 @@
         <v>6402</v>
       </c>
       <c r="B56" t="s">
-        <v>369</v>
+        <v>354</v>
       </c>
       <c r="C56" t="s">
-        <v>370</v>
+        <v>355</v>
       </c>
       <c r="D56">
         <v>2</v>
@@ -3952,10 +3907,10 @@
         <v>6403</v>
       </c>
       <c r="B57" t="s">
-        <v>371</v>
+        <v>356</v>
       </c>
       <c r="C57" t="s">
-        <v>372</v>
+        <v>357</v>
       </c>
       <c r="D57">
         <v>2</v>
@@ -3982,10 +3937,10 @@
         <v>6404</v>
       </c>
       <c r="B58" t="s">
-        <v>373</v>
+        <v>358</v>
       </c>
       <c r="C58" t="s">
-        <v>374</v>
+        <v>359</v>
       </c>
       <c r="D58">
         <v>2</v>
@@ -4012,10 +3967,10 @@
         <v>6405</v>
       </c>
       <c r="B59" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="C59" t="s">
-        <v>376</v>
+        <v>361</v>
       </c>
       <c r="D59">
         <v>2</v>
@@ -4042,10 +3997,10 @@
         <v>6406</v>
       </c>
       <c r="B60" t="s">
-        <v>377</v>
+        <v>362</v>
       </c>
       <c r="C60" t="s">
-        <v>378</v>
+        <v>363</v>
       </c>
       <c r="D60">
         <v>2</v>
@@ -4072,10 +4027,10 @@
         <v>6407</v>
       </c>
       <c r="B61" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
       <c r="C61" t="s">
-        <v>380</v>
+        <v>365</v>
       </c>
       <c r="D61">
         <v>2</v>
@@ -4102,10 +4057,10 @@
         <v>6408</v>
       </c>
       <c r="B62" t="s">
-        <v>381</v>
+        <v>366</v>
       </c>
       <c r="C62" t="s">
-        <v>382</v>
+        <v>367</v>
       </c>
       <c r="D62">
         <v>2</v>
@@ -4132,10 +4087,10 @@
         <v>6409</v>
       </c>
       <c r="B63" t="s">
-        <v>383</v>
+        <v>368</v>
       </c>
       <c r="C63" t="s">
-        <v>384</v>
+        <v>369</v>
       </c>
       <c r="D63">
         <v>2</v>
@@ -4162,10 +4117,10 @@
         <v>6410</v>
       </c>
       <c r="B64" t="s">
-        <v>385</v>
+        <v>370</v>
       </c>
       <c r="C64" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="D64">
         <v>2</v>
@@ -4192,10 +4147,10 @@
         <v>6411</v>
       </c>
       <c r="B65" t="s">
-        <v>387</v>
+        <v>372</v>
       </c>
       <c r="C65" t="s">
-        <v>388</v>
+        <v>373</v>
       </c>
       <c r="D65">
         <v>2</v>
@@ -4222,10 +4177,10 @@
         <v>6412</v>
       </c>
       <c r="B66" t="s">
-        <v>389</v>
+        <v>374</v>
       </c>
       <c r="C66" t="s">
-        <v>390</v>
+        <v>375</v>
       </c>
       <c r="D66">
         <v>3</v>
@@ -4252,10 +4207,10 @@
         <v>6413</v>
       </c>
       <c r="B67" t="s">
-        <v>391</v>
+        <v>376</v>
       </c>
       <c r="C67" t="s">
-        <v>392</v>
+        <v>377</v>
       </c>
       <c r="D67">
         <v>3</v>
@@ -4282,10 +4237,10 @@
         <v>6414</v>
       </c>
       <c r="B68" t="s">
-        <v>393</v>
+        <v>378</v>
       </c>
       <c r="C68" t="s">
-        <v>394</v>
+        <v>379</v>
       </c>
       <c r="D68">
         <v>3</v>
@@ -4312,10 +4267,10 @@
         <v>6415</v>
       </c>
       <c r="B69" t="s">
-        <v>395</v>
+        <v>380</v>
       </c>
       <c r="C69" t="s">
-        <v>396</v>
+        <v>381</v>
       </c>
       <c r="D69">
         <v>3</v>
@@ -4342,10 +4297,10 @@
         <v>6416</v>
       </c>
       <c r="B70" t="s">
-        <v>397</v>
+        <v>382</v>
       </c>
       <c r="C70" t="s">
-        <v>398</v>
+        <v>383</v>
       </c>
       <c r="D70">
         <v>3</v>
@@ -4372,10 +4327,10 @@
         <v>6417</v>
       </c>
       <c r="B71" t="s">
-        <v>399</v>
+        <v>384</v>
       </c>
       <c r="C71" t="s">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="D71">
         <v>3</v>
@@ -4402,10 +4357,10 @@
         <v>6418</v>
       </c>
       <c r="B72" t="s">
-        <v>401</v>
+        <v>386</v>
       </c>
       <c r="C72" t="s">
-        <v>402</v>
+        <v>387</v>
       </c>
       <c r="D72">
         <v>3</v>
@@ -4432,10 +4387,10 @@
         <v>6419</v>
       </c>
       <c r="B73" t="s">
-        <v>403</v>
+        <v>388</v>
       </c>
       <c r="C73" t="s">
-        <v>404</v>
+        <v>389</v>
       </c>
       <c r="D73">
         <v>3</v>
@@ -4462,10 +4417,10 @@
         <v>6420</v>
       </c>
       <c r="B74" t="s">
-        <v>405</v>
+        <v>390</v>
       </c>
       <c r="C74" t="s">
-        <v>406</v>
+        <v>391</v>
       </c>
       <c r="D74">
         <v>3</v>
@@ -4492,10 +4447,10 @@
         <v>6421</v>
       </c>
       <c r="B75" t="s">
-        <v>407</v>
+        <v>392</v>
       </c>
       <c r="C75" t="s">
-        <v>408</v>
+        <v>393</v>
       </c>
       <c r="D75">
         <v>3</v>
@@ -4522,10 +4477,10 @@
         <v>6422</v>
       </c>
       <c r="B76" t="s">
-        <v>409</v>
+        <v>394</v>
       </c>
       <c r="C76" t="s">
-        <v>410</v>
+        <v>395</v>
       </c>
       <c r="D76">
         <v>4</v>
@@ -4552,10 +4507,10 @@
         <v>6423</v>
       </c>
       <c r="B77" t="s">
-        <v>411</v>
+        <v>396</v>
       </c>
       <c r="C77" t="s">
-        <v>412</v>
+        <v>397</v>
       </c>
       <c r="D77">
         <v>4</v>
@@ -4582,10 +4537,10 @@
         <v>6424</v>
       </c>
       <c r="B78" t="s">
-        <v>413</v>
+        <v>398</v>
       </c>
       <c r="C78" t="s">
-        <v>414</v>
+        <v>399</v>
       </c>
       <c r="D78">
         <v>4</v>
@@ -4601,7 +4556,7 @@
         <v>147</v>
       </c>
       <c r="H78" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I78">
         <v>2</v>
@@ -4612,10 +4567,10 @@
         <v>6425</v>
       </c>
       <c r="B79" t="s">
-        <v>415</v>
+        <v>400</v>
       </c>
       <c r="C79" t="s">
-        <v>416</v>
+        <v>401</v>
       </c>
       <c r="D79">
         <v>4</v>
@@ -4631,7 +4586,7 @@
         <v>147</v>
       </c>
       <c r="H79" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I79">
         <v>2</v>
@@ -4642,10 +4597,10 @@
         <v>6426</v>
       </c>
       <c r="B80" t="s">
-        <v>417</v>
+        <v>402</v>
       </c>
       <c r="C80" t="s">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="D80">
         <v>4</v>
@@ -4661,7 +4616,7 @@
         <v>147</v>
       </c>
       <c r="H80" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I80">
         <v>2</v>
@@ -4672,10 +4627,10 @@
         <v>6427</v>
       </c>
       <c r="B81" t="s">
-        <v>419</v>
+        <v>404</v>
       </c>
       <c r="C81" t="s">
-        <v>420</v>
+        <v>405</v>
       </c>
       <c r="D81">
         <v>4</v>
@@ -4691,7 +4646,7 @@
         <v>147</v>
       </c>
       <c r="H81" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I81">
         <v>2</v>
@@ -4702,10 +4657,10 @@
         <v>6428</v>
       </c>
       <c r="B82" t="s">
-        <v>421</v>
+        <v>406</v>
       </c>
       <c r="C82" t="s">
-        <v>422</v>
+        <v>407</v>
       </c>
       <c r="D82">
         <v>4</v>
@@ -4721,7 +4676,7 @@
         <v>147</v>
       </c>
       <c r="H82" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I82">
         <v>2</v>
@@ -4732,10 +4687,10 @@
         <v>6429</v>
       </c>
       <c r="B83" t="s">
-        <v>423</v>
+        <v>408</v>
       </c>
       <c r="C83" t="s">
-        <v>424</v>
+        <v>409</v>
       </c>
       <c r="D83">
         <v>4</v>
@@ -4751,7 +4706,7 @@
         <v>147</v>
       </c>
       <c r="H83" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I83">
         <v>2</v>
@@ -4762,10 +4717,10 @@
         <v>6430</v>
       </c>
       <c r="B84" t="s">
-        <v>425</v>
+        <v>410</v>
       </c>
       <c r="C84" t="s">
-        <v>426</v>
+        <v>411</v>
       </c>
       <c r="D84">
         <v>4</v>
@@ -4781,7 +4736,7 @@
         <v>147</v>
       </c>
       <c r="H84" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I84">
         <v>2</v>
@@ -4792,10 +4747,10 @@
         <v>6431</v>
       </c>
       <c r="B85" t="s">
-        <v>427</v>
+        <v>412</v>
       </c>
       <c r="C85" t="s">
-        <v>428</v>
+        <v>413</v>
       </c>
       <c r="D85">
         <v>4</v>
@@ -4822,10 +4777,10 @@
         <v>6432</v>
       </c>
       <c r="B86" t="s">
-        <v>429</v>
+        <v>414</v>
       </c>
       <c r="C86" t="s">
-        <v>430</v>
+        <v>415</v>
       </c>
       <c r="D86">
         <v>4</v>
@@ -4852,10 +4807,10 @@
         <v>6302</v>
       </c>
       <c r="B87" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="C87" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="D87">
         <v>1</v>
@@ -4882,7 +4837,7 @@
         <v>6303</v>
       </c>
       <c r="B88" t="s">
-        <v>354</v>
+        <v>339</v>
       </c>
       <c r="C88" t="s">
         <v>9</v>
@@ -4912,10 +4867,10 @@
         <v>6304</v>
       </c>
       <c r="B89" t="s">
-        <v>355</v>
+        <v>340</v>
       </c>
       <c r="C89" t="s">
-        <v>356</v>
+        <v>341</v>
       </c>
       <c r="D89">
         <v>1</v>
@@ -4942,10 +4897,10 @@
         <v>6305</v>
       </c>
       <c r="B90" t="s">
-        <v>365</v>
+        <v>350</v>
       </c>
       <c r="C90" t="s">
-        <v>366</v>
+        <v>351</v>
       </c>
       <c r="D90">
         <v>1</v>
@@ -4972,10 +4927,10 @@
         <v>6306</v>
       </c>
       <c r="B91" t="s">
-        <v>357</v>
+        <v>342</v>
       </c>
       <c r="C91" t="s">
-        <v>358</v>
+        <v>343</v>
       </c>
       <c r="D91">
         <v>1</v>
@@ -5002,10 +4957,10 @@
         <v>6307</v>
       </c>
       <c r="B92" t="s">
-        <v>361</v>
+        <v>346</v>
       </c>
       <c r="C92" t="s">
-        <v>362</v>
+        <v>347</v>
       </c>
       <c r="D92">
         <v>1</v>
@@ -5062,10 +5017,10 @@
         <v>6309</v>
       </c>
       <c r="B94" t="s">
-        <v>363</v>
+        <v>348</v>
       </c>
       <c r="C94" t="s">
-        <v>364</v>
+        <v>349</v>
       </c>
       <c r="D94">
         <v>1</v>
@@ -5092,10 +5047,10 @@
         <v>6310</v>
       </c>
       <c r="B95" t="s">
-        <v>359</v>
+        <v>344</v>
       </c>
       <c r="C95" t="s">
-        <v>360</v>
+        <v>345</v>
       </c>
       <c r="D95">
         <v>1</v>
@@ -5122,10 +5077,10 @@
         <v>6311</v>
       </c>
       <c r="B96" t="s">
-        <v>367</v>
+        <v>352</v>
       </c>
       <c r="C96" t="s">
-        <v>368</v>
+        <v>353</v>
       </c>
       <c r="D96">
         <v>1</v>
@@ -5152,10 +5107,10 @@
         <v>6312</v>
       </c>
       <c r="B97" t="s">
-        <v>431</v>
+        <v>416</v>
       </c>
       <c r="C97" t="s">
-        <v>432</v>
+        <v>417</v>
       </c>
       <c r="D97">
         <v>2</v>
@@ -5182,10 +5137,10 @@
         <v>6313</v>
       </c>
       <c r="B98" t="s">
-        <v>373</v>
+        <v>358</v>
       </c>
       <c r="C98" t="s">
-        <v>374</v>
+        <v>359</v>
       </c>
       <c r="D98">
         <v>2</v>
@@ -5212,10 +5167,10 @@
         <v>6314</v>
       </c>
       <c r="B99" t="s">
-        <v>377</v>
+        <v>362</v>
       </c>
       <c r="C99" t="s">
-        <v>433</v>
+        <v>418</v>
       </c>
       <c r="D99">
         <v>2</v>
@@ -5242,10 +5197,10 @@
         <v>6315</v>
       </c>
       <c r="B100" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
       <c r="C100" t="s">
-        <v>380</v>
+        <v>365</v>
       </c>
       <c r="D100">
         <v>2</v>
@@ -5272,10 +5227,10 @@
         <v>6316</v>
       </c>
       <c r="B101" t="s">
-        <v>385</v>
+        <v>370</v>
       </c>
       <c r="C101" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="D101">
         <v>2</v>
@@ -5302,10 +5257,10 @@
         <v>6317</v>
       </c>
       <c r="B102" t="s">
-        <v>434</v>
+        <v>419</v>
       </c>
       <c r="C102" t="s">
-        <v>435</v>
+        <v>420</v>
       </c>
       <c r="D102">
         <v>2</v>
@@ -5332,10 +5287,10 @@
         <v>6318</v>
       </c>
       <c r="B103" t="s">
-        <v>381</v>
+        <v>366</v>
       </c>
       <c r="C103" t="s">
-        <v>382</v>
+        <v>367</v>
       </c>
       <c r="D103">
         <v>2</v>
@@ -5362,10 +5317,10 @@
         <v>6319</v>
       </c>
       <c r="B104" t="s">
-        <v>383</v>
+        <v>368</v>
       </c>
       <c r="C104" t="s">
-        <v>384</v>
+        <v>369</v>
       </c>
       <c r="D104">
         <v>2</v>
@@ -5392,10 +5347,10 @@
         <v>6320</v>
       </c>
       <c r="B105" t="s">
-        <v>371</v>
+        <v>356</v>
       </c>
       <c r="C105" t="s">
-        <v>372</v>
+        <v>357</v>
       </c>
       <c r="D105">
         <v>2</v>
@@ -5422,10 +5377,10 @@
         <v>6321</v>
       </c>
       <c r="B106" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="C106" t="s">
-        <v>303</v>
+        <v>288</v>
       </c>
       <c r="D106">
         <v>2</v>
@@ -5452,10 +5407,10 @@
         <v>6322</v>
       </c>
       <c r="B107" t="s">
-        <v>407</v>
+        <v>392</v>
       </c>
       <c r="C107" t="s">
-        <v>408</v>
+        <v>393</v>
       </c>
       <c r="D107">
         <v>3</v>
@@ -5482,10 +5437,10 @@
         <v>6323</v>
       </c>
       <c r="B108" t="s">
-        <v>436</v>
+        <v>421</v>
       </c>
       <c r="C108" t="s">
-        <v>437</v>
+        <v>422</v>
       </c>
       <c r="D108">
         <v>3</v>
@@ -5512,10 +5467,10 @@
         <v>6324</v>
       </c>
       <c r="B109" t="s">
-        <v>438</v>
+        <v>423</v>
       </c>
       <c r="C109" t="s">
-        <v>439</v>
+        <v>424</v>
       </c>
       <c r="D109">
         <v>3</v>
@@ -5542,10 +5497,10 @@
         <v>6325</v>
       </c>
       <c r="B110" t="s">
-        <v>440</v>
+        <v>425</v>
       </c>
       <c r="C110" t="s">
-        <v>441</v>
+        <v>426</v>
       </c>
       <c r="D110">
         <v>3</v>
@@ -5572,10 +5527,10 @@
         <v>6326</v>
       </c>
       <c r="B111" t="s">
-        <v>442</v>
+        <v>427</v>
       </c>
       <c r="C111" t="s">
-        <v>443</v>
+        <v>428</v>
       </c>
       <c r="D111">
         <v>3</v>
@@ -5602,10 +5557,10 @@
         <v>6327</v>
       </c>
       <c r="B112" t="s">
-        <v>444</v>
+        <v>429</v>
       </c>
       <c r="C112" t="s">
-        <v>445</v>
+        <v>430</v>
       </c>
       <c r="D112">
         <v>3</v>
@@ -5632,10 +5587,10 @@
         <v>6328</v>
       </c>
       <c r="B113" t="s">
-        <v>446</v>
+        <v>431</v>
       </c>
       <c r="C113" t="s">
-        <v>447</v>
+        <v>432</v>
       </c>
       <c r="D113">
         <v>3</v>
@@ -5662,10 +5617,10 @@
         <v>6329</v>
       </c>
       <c r="B114" t="s">
-        <v>448</v>
+        <v>433</v>
       </c>
       <c r="C114" t="s">
-        <v>449</v>
+        <v>434</v>
       </c>
       <c r="D114">
         <v>3</v>
@@ -5692,10 +5647,10 @@
         <v>6330</v>
       </c>
       <c r="B115" t="s">
-        <v>450</v>
+        <v>435</v>
       </c>
       <c r="C115" t="s">
-        <v>451</v>
+        <v>436</v>
       </c>
       <c r="D115">
         <v>3</v>
@@ -5722,10 +5677,10 @@
         <v>6331</v>
       </c>
       <c r="B116" t="s">
-        <v>452</v>
+        <v>437</v>
       </c>
       <c r="C116" t="s">
-        <v>453</v>
+        <v>438</v>
       </c>
       <c r="D116">
         <v>3</v>
@@ -5752,10 +5707,10 @@
         <v>6332</v>
       </c>
       <c r="B117" t="s">
-        <v>454</v>
+        <v>439</v>
       </c>
       <c r="C117" t="s">
-        <v>455</v>
+        <v>440</v>
       </c>
       <c r="D117">
         <v>4</v>
@@ -5782,10 +5737,10 @@
         <v>6333</v>
       </c>
       <c r="B118" t="s">
-        <v>456</v>
+        <v>441</v>
       </c>
       <c r="C118" t="s">
-        <v>457</v>
+        <v>442</v>
       </c>
       <c r="D118">
         <v>4</v>
@@ -5812,10 +5767,10 @@
         <v>6334</v>
       </c>
       <c r="B119" t="s">
-        <v>458</v>
+        <v>443</v>
       </c>
       <c r="C119" t="s">
-        <v>459</v>
+        <v>444</v>
       </c>
       <c r="D119">
         <v>4</v>
@@ -5842,10 +5797,10 @@
         <v>6335</v>
       </c>
       <c r="B120" t="s">
-        <v>460</v>
+        <v>445</v>
       </c>
       <c r="C120" t="s">
-        <v>461</v>
+        <v>446</v>
       </c>
       <c r="D120">
         <v>4</v>
@@ -5872,10 +5827,10 @@
         <v>6336</v>
       </c>
       <c r="B121" t="s">
-        <v>411</v>
+        <v>396</v>
       </c>
       <c r="C121" t="s">
-        <v>412</v>
+        <v>397</v>
       </c>
       <c r="D121">
         <v>4</v>
@@ -5902,10 +5857,10 @@
         <v>8507</v>
       </c>
       <c r="B122" t="s">
-        <v>462</v>
+        <v>447</v>
       </c>
       <c r="C122" t="s">
-        <v>463</v>
+        <v>448</v>
       </c>
       <c r="D122">
         <v>4</v>
@@ -5921,7 +5876,7 @@
         <v>166</v>
       </c>
       <c r="H122" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I122">
         <v>2</v>
@@ -5932,10 +5887,10 @@
         <v>6338</v>
       </c>
       <c r="B123" t="s">
-        <v>464</v>
+        <v>449</v>
       </c>
       <c r="C123" t="s">
-        <v>465</v>
+        <v>450</v>
       </c>
       <c r="D123">
         <v>4</v>
@@ -5951,7 +5906,7 @@
         <v>166</v>
       </c>
       <c r="H123" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I123">
         <v>2</v>
@@ -5962,10 +5917,10 @@
         <v>6339</v>
       </c>
       <c r="B124" t="s">
-        <v>466</v>
+        <v>451</v>
       </c>
       <c r="C124" t="s">
-        <v>467</v>
+        <v>452</v>
       </c>
       <c r="D124">
         <v>4</v>
@@ -5981,7 +5936,7 @@
         <v>166</v>
       </c>
       <c r="H124" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I124">
         <v>2</v>
@@ -5992,10 +5947,10 @@
         <v>6340</v>
       </c>
       <c r="B125" t="s">
-        <v>468</v>
+        <v>453</v>
       </c>
       <c r="C125" t="s">
-        <v>469</v>
+        <v>454</v>
       </c>
       <c r="D125">
         <v>4</v>
@@ -6011,7 +5966,7 @@
         <v>166</v>
       </c>
       <c r="H125" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I125">
         <v>2</v>
@@ -6022,10 +5977,10 @@
         <v>6341</v>
       </c>
       <c r="B126" t="s">
-        <v>470</v>
+        <v>455</v>
       </c>
       <c r="C126" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="D126">
         <v>4</v>
@@ -6041,7 +5996,7 @@
         <v>166</v>
       </c>
       <c r="H126" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I126">
         <v>2</v>
@@ -6052,10 +6007,10 @@
         <v>9115</v>
       </c>
       <c r="B127" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="C127" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="D127">
         <v>1</v>
@@ -6082,7 +6037,7 @@
         <v>9116</v>
       </c>
       <c r="B128" t="s">
-        <v>355</v>
+        <v>340</v>
       </c>
       <c r="C128" t="s">
         <v>18</v>
@@ -6112,10 +6067,10 @@
         <v>9117</v>
       </c>
       <c r="B129" t="s">
-        <v>471</v>
+        <v>456</v>
       </c>
       <c r="C129" t="s">
-        <v>472</v>
+        <v>457</v>
       </c>
       <c r="D129">
         <v>1</v>
@@ -6172,10 +6127,10 @@
         <v>9119</v>
       </c>
       <c r="B131" t="s">
-        <v>365</v>
+        <v>350</v>
       </c>
       <c r="C131" t="s">
-        <v>366</v>
+        <v>351</v>
       </c>
       <c r="D131">
         <v>1</v>
@@ -6202,7 +6157,7 @@
         <v>9120</v>
       </c>
       <c r="B132" t="s">
-        <v>354</v>
+        <v>339</v>
       </c>
       <c r="C132" t="s">
         <v>9</v>
@@ -6232,10 +6187,10 @@
         <v>9121</v>
       </c>
       <c r="B133" t="s">
-        <v>363</v>
+        <v>348</v>
       </c>
       <c r="C133" t="s">
-        <v>364</v>
+        <v>349</v>
       </c>
       <c r="D133">
         <v>1</v>
@@ -6262,10 +6217,10 @@
         <v>9122</v>
       </c>
       <c r="B134" t="s">
-        <v>361</v>
+        <v>346</v>
       </c>
       <c r="C134" t="s">
-        <v>362</v>
+        <v>347</v>
       </c>
       <c r="D134">
         <v>1</v>
@@ -6292,10 +6247,10 @@
         <v>9123</v>
       </c>
       <c r="B135" t="s">
-        <v>367</v>
+        <v>352</v>
       </c>
       <c r="C135" t="s">
-        <v>368</v>
+        <v>353</v>
       </c>
       <c r="D135">
         <v>1</v>
@@ -6322,10 +6277,10 @@
         <v>9124</v>
       </c>
       <c r="B136" t="s">
-        <v>359</v>
+        <v>344</v>
       </c>
       <c r="C136" t="s">
-        <v>360</v>
+        <v>345</v>
       </c>
       <c r="D136">
         <v>1</v>
@@ -6352,10 +6307,10 @@
         <v>9125</v>
       </c>
       <c r="B137" t="s">
-        <v>473</v>
+        <v>458</v>
       </c>
       <c r="C137" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="D137">
         <v>2</v>
@@ -6382,10 +6337,10 @@
         <v>9126</v>
       </c>
       <c r="B138" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="C138" t="s">
-        <v>303</v>
+        <v>288</v>
       </c>
       <c r="D138">
         <v>2</v>
@@ -6412,10 +6367,10 @@
         <v>9127</v>
       </c>
       <c r="B139" t="s">
-        <v>474</v>
+        <v>459</v>
       </c>
       <c r="C139" t="s">
-        <v>378</v>
+        <v>363</v>
       </c>
       <c r="D139">
         <v>2</v>
@@ -6442,10 +6397,10 @@
         <v>9128</v>
       </c>
       <c r="B140" t="s">
-        <v>475</v>
+        <v>460</v>
       </c>
       <c r="C140" t="s">
-        <v>374</v>
+        <v>359</v>
       </c>
       <c r="D140">
         <v>2</v>
@@ -6472,10 +6427,10 @@
         <v>9129</v>
       </c>
       <c r="B141" t="s">
-        <v>476</v>
+        <v>461</v>
       </c>
       <c r="C141" t="s">
-        <v>380</v>
+        <v>365</v>
       </c>
       <c r="D141">
         <v>2</v>
@@ -6502,10 +6457,10 @@
         <v>9130</v>
       </c>
       <c r="B142" t="s">
-        <v>434</v>
+        <v>419</v>
       </c>
       <c r="C142" t="s">
-        <v>435</v>
+        <v>420</v>
       </c>
       <c r="D142">
         <v>2</v>
@@ -6532,10 +6487,10 @@
         <v>9131</v>
       </c>
       <c r="B143" t="s">
-        <v>371</v>
+        <v>356</v>
       </c>
       <c r="C143" t="s">
-        <v>372</v>
+        <v>357</v>
       </c>
       <c r="D143">
         <v>2</v>
@@ -6562,10 +6517,10 @@
         <v>9132</v>
       </c>
       <c r="B144" t="s">
-        <v>477</v>
+        <v>462</v>
       </c>
       <c r="C144" t="s">
-        <v>370</v>
+        <v>355</v>
       </c>
       <c r="D144">
         <v>2</v>
@@ -6592,10 +6547,10 @@
         <v>9133</v>
       </c>
       <c r="B145" t="s">
-        <v>478</v>
+        <v>463</v>
       </c>
       <c r="C145" t="s">
-        <v>384</v>
+        <v>369</v>
       </c>
       <c r="D145">
         <v>2</v>
@@ -6622,10 +6577,10 @@
         <v>9134</v>
       </c>
       <c r="B146" t="s">
-        <v>381</v>
+        <v>366</v>
       </c>
       <c r="C146" t="s">
-        <v>382</v>
+        <v>367</v>
       </c>
       <c r="D146">
         <v>2</v>
@@ -6652,10 +6607,10 @@
         <v>9135</v>
       </c>
       <c r="B147" t="s">
-        <v>479</v>
+        <v>464</v>
       </c>
       <c r="C147" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D147">
         <v>3</v>
@@ -6682,10 +6637,10 @@
         <v>9136</v>
       </c>
       <c r="B148" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
       <c r="C148" t="s">
-        <v>482</v>
+        <v>467</v>
       </c>
       <c r="D148">
         <v>3</v>
@@ -6712,10 +6667,10 @@
         <v>9137</v>
       </c>
       <c r="B149" t="s">
-        <v>483</v>
+        <v>468</v>
       </c>
       <c r="C149" t="s">
-        <v>484</v>
+        <v>469</v>
       </c>
       <c r="D149">
         <v>3</v>
@@ -6742,10 +6697,10 @@
         <v>9138</v>
       </c>
       <c r="B150" t="s">
-        <v>485</v>
+        <v>470</v>
       </c>
       <c r="C150" t="s">
-        <v>486</v>
+        <v>471</v>
       </c>
       <c r="D150">
         <v>3</v>
@@ -6772,10 +6727,10 @@
         <v>9139</v>
       </c>
       <c r="B151" t="s">
-        <v>487</v>
+        <v>472</v>
       </c>
       <c r="C151" t="s">
-        <v>408</v>
+        <v>393</v>
       </c>
       <c r="D151">
         <v>3</v>
@@ -6802,10 +6757,10 @@
         <v>9140</v>
       </c>
       <c r="B152" t="s">
-        <v>488</v>
+        <v>473</v>
       </c>
       <c r="C152" t="s">
-        <v>489</v>
+        <v>474</v>
       </c>
       <c r="D152">
         <v>3</v>
@@ -6832,10 +6787,10 @@
         <v>9141</v>
       </c>
       <c r="B153" t="s">
-        <v>490</v>
+        <v>475</v>
       </c>
       <c r="C153" t="s">
-        <v>491</v>
+        <v>476</v>
       </c>
       <c r="D153">
         <v>3</v>
@@ -6862,10 +6817,10 @@
         <v>9142</v>
       </c>
       <c r="B154" t="s">
-        <v>492</v>
+        <v>477</v>
       </c>
       <c r="C154" t="s">
-        <v>493</v>
+        <v>478</v>
       </c>
       <c r="D154">
         <v>3</v>
@@ -6892,10 +6847,10 @@
         <v>9143</v>
       </c>
       <c r="B155" t="s">
-        <v>494</v>
+        <v>479</v>
       </c>
       <c r="C155" t="s">
-        <v>495</v>
+        <v>480</v>
       </c>
       <c r="D155">
         <v>3</v>
@@ -6922,10 +6877,10 @@
         <v>9144</v>
       </c>
       <c r="B156" t="s">
-        <v>496</v>
+        <v>481</v>
       </c>
       <c r="C156" t="s">
-        <v>497</v>
+        <v>482</v>
       </c>
       <c r="D156">
         <v>3</v>
@@ -6952,10 +6907,10 @@
         <v>9145</v>
       </c>
       <c r="B157" t="s">
-        <v>411</v>
+        <v>396</v>
       </c>
       <c r="C157" t="s">
-        <v>412</v>
+        <v>397</v>
       </c>
       <c r="D157">
         <v>4</v>
@@ -6982,10 +6937,10 @@
         <v>9146</v>
       </c>
       <c r="B158" t="s">
-        <v>310</v>
+        <v>295</v>
       </c>
       <c r="C158" t="s">
-        <v>498</v>
+        <v>483</v>
       </c>
       <c r="D158">
         <v>4</v>
@@ -7012,10 +6967,10 @@
         <v>9147</v>
       </c>
       <c r="B159" t="s">
-        <v>499</v>
+        <v>484</v>
       </c>
       <c r="C159" t="s">
-        <v>500</v>
+        <v>485</v>
       </c>
       <c r="D159">
         <v>4</v>
@@ -7042,10 +6997,10 @@
         <v>9148</v>
       </c>
       <c r="B160" t="s">
-        <v>501</v>
+        <v>486</v>
       </c>
       <c r="C160" t="s">
-        <v>502</v>
+        <v>487</v>
       </c>
       <c r="D160">
         <v>4</v>
@@ -7072,10 +7027,10 @@
         <v>9149</v>
       </c>
       <c r="B161" t="s">
-        <v>503</v>
+        <v>488</v>
       </c>
       <c r="C161" t="s">
-        <v>504</v>
+        <v>489</v>
       </c>
       <c r="D161">
         <v>4</v>
@@ -7102,10 +7057,10 @@
         <v>9151</v>
       </c>
       <c r="B162" t="s">
-        <v>505</v>
+        <v>490</v>
       </c>
       <c r="C162" t="s">
-        <v>506</v>
+        <v>491</v>
       </c>
       <c r="D162">
         <v>4</v>
@@ -7121,7 +7076,7 @@
         <v>291</v>
       </c>
       <c r="H162" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I162">
         <v>2</v>
@@ -7132,10 +7087,10 @@
         <v>9152</v>
       </c>
       <c r="B163" t="s">
-        <v>507</v>
+        <v>492</v>
       </c>
       <c r="C163" t="s">
-        <v>508</v>
+        <v>493</v>
       </c>
       <c r="D163">
         <v>4</v>
@@ -7151,7 +7106,7 @@
         <v>291</v>
       </c>
       <c r="H163" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I163">
         <v>2</v>
@@ -7162,10 +7117,10 @@
         <v>9153</v>
       </c>
       <c r="B164" t="s">
-        <v>509</v>
+        <v>494</v>
       </c>
       <c r="C164" t="s">
-        <v>510</v>
+        <v>495</v>
       </c>
       <c r="D164">
         <v>4</v>
@@ -7181,7 +7136,7 @@
         <v>291</v>
       </c>
       <c r="H164" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I164">
         <v>2</v>
@@ -7192,10 +7147,10 @@
         <v>7711</v>
       </c>
       <c r="B165" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="C165" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="D165">
         <v>1</v>
@@ -7222,10 +7177,10 @@
         <v>7712</v>
       </c>
       <c r="B166" t="s">
-        <v>354</v>
+        <v>339</v>
       </c>
       <c r="C166" t="s">
-        <v>511</v>
+        <v>496</v>
       </c>
       <c r="D166">
         <v>1</v>
@@ -7252,10 +7207,10 @@
         <v>7713</v>
       </c>
       <c r="B167" t="s">
-        <v>355</v>
+        <v>340</v>
       </c>
       <c r="C167" t="s">
-        <v>512</v>
+        <v>497</v>
       </c>
       <c r="D167">
         <v>1</v>
@@ -7282,10 +7237,10 @@
         <v>7714</v>
       </c>
       <c r="B168" t="s">
-        <v>365</v>
+        <v>350</v>
       </c>
       <c r="C168" t="s">
-        <v>366</v>
+        <v>351</v>
       </c>
       <c r="D168">
         <v>1</v>
@@ -7312,10 +7267,10 @@
         <v>7715</v>
       </c>
       <c r="B169" t="s">
-        <v>513</v>
+        <v>498</v>
       </c>
       <c r="C169" t="s">
-        <v>514</v>
+        <v>499</v>
       </c>
       <c r="D169">
         <v>1</v>
@@ -7342,10 +7297,10 @@
         <v>7716</v>
       </c>
       <c r="B170" t="s">
-        <v>361</v>
+        <v>346</v>
       </c>
       <c r="C170" t="s">
-        <v>362</v>
+        <v>347</v>
       </c>
       <c r="D170">
         <v>1</v>
@@ -7402,10 +7357,10 @@
         <v>7718</v>
       </c>
       <c r="B172" t="s">
-        <v>363</v>
+        <v>348</v>
       </c>
       <c r="C172" t="s">
-        <v>515</v>
+        <v>500</v>
       </c>
       <c r="D172">
         <v>1</v>
@@ -7432,10 +7387,10 @@
         <v>7719</v>
       </c>
       <c r="B173" t="s">
-        <v>516</v>
+        <v>501</v>
       </c>
       <c r="C173" t="s">
-        <v>517</v>
+        <v>502</v>
       </c>
       <c r="D173">
         <v>1</v>
@@ -7462,10 +7417,10 @@
         <v>7720</v>
       </c>
       <c r="B174" t="s">
-        <v>367</v>
+        <v>352</v>
       </c>
       <c r="C174" t="s">
-        <v>368</v>
+        <v>353</v>
       </c>
       <c r="D174">
         <v>1</v>
@@ -7492,10 +7447,10 @@
         <v>7721</v>
       </c>
       <c r="B175" t="s">
-        <v>434</v>
+        <v>419</v>
       </c>
       <c r="C175" t="s">
-        <v>435</v>
+        <v>420</v>
       </c>
       <c r="D175">
         <v>1</v>
@@ -7522,10 +7477,10 @@
         <v>7722</v>
       </c>
       <c r="B176" t="s">
-        <v>431</v>
+        <v>416</v>
       </c>
       <c r="C176" t="s">
-        <v>518</v>
+        <v>503</v>
       </c>
       <c r="D176">
         <v>2</v>
@@ -7552,10 +7507,10 @@
         <v>7723</v>
       </c>
       <c r="B177" t="s">
-        <v>373</v>
+        <v>358</v>
       </c>
       <c r="C177" t="s">
-        <v>374</v>
+        <v>359</v>
       </c>
       <c r="D177">
         <v>2</v>
@@ -7582,10 +7537,10 @@
         <v>7724</v>
       </c>
       <c r="B178" t="s">
-        <v>377</v>
+        <v>362</v>
       </c>
       <c r="C178" t="s">
-        <v>519</v>
+        <v>504</v>
       </c>
       <c r="D178">
         <v>2</v>
@@ -7612,10 +7567,10 @@
         <v>7725</v>
       </c>
       <c r="B179" t="s">
-        <v>371</v>
+        <v>356</v>
       </c>
       <c r="C179" t="s">
-        <v>372</v>
+        <v>357</v>
       </c>
       <c r="D179">
         <v>2</v>
@@ -7642,10 +7597,10 @@
         <v>7726</v>
       </c>
       <c r="B180" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="C180" t="s">
-        <v>520</v>
+        <v>505</v>
       </c>
       <c r="D180">
         <v>2</v>
@@ -7672,10 +7627,10 @@
         <v>7727</v>
       </c>
       <c r="B181" t="s">
-        <v>468</v>
+        <v>453</v>
       </c>
       <c r="C181" t="s">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="D181">
         <v>2</v>
@@ -7702,10 +7657,10 @@
         <v>7728</v>
       </c>
       <c r="B182" t="s">
-        <v>387</v>
+        <v>372</v>
       </c>
       <c r="C182" t="s">
-        <v>388</v>
+        <v>373</v>
       </c>
       <c r="D182">
         <v>2</v>
@@ -7732,10 +7687,10 @@
         <v>7729</v>
       </c>
       <c r="B183" t="s">
-        <v>381</v>
+        <v>366</v>
       </c>
       <c r="C183" t="s">
-        <v>382</v>
+        <v>367</v>
       </c>
       <c r="D183">
         <v>2</v>
@@ -7762,10 +7717,10 @@
         <v>7730</v>
       </c>
       <c r="B184" t="s">
-        <v>383</v>
+        <v>368</v>
       </c>
       <c r="C184" t="s">
-        <v>384</v>
+        <v>369</v>
       </c>
       <c r="D184">
         <v>2</v>
@@ -7792,10 +7747,10 @@
         <v>7731</v>
       </c>
       <c r="B185" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
       <c r="C185" t="s">
-        <v>380</v>
+        <v>365</v>
       </c>
       <c r="D185">
         <v>2</v>
@@ -7822,10 +7777,10 @@
         <v>7732</v>
       </c>
       <c r="B186" t="s">
-        <v>521</v>
+        <v>506</v>
       </c>
       <c r="C186" t="s">
-        <v>386</v>
+        <v>371</v>
       </c>
       <c r="D186">
         <v>2</v>
@@ -7852,10 +7807,10 @@
         <v>7733</v>
       </c>
       <c r="B187" t="s">
-        <v>436</v>
+        <v>421</v>
       </c>
       <c r="C187" t="s">
-        <v>360</v>
+        <v>345</v>
       </c>
       <c r="D187">
         <v>3</v>
@@ -7882,10 +7837,10 @@
         <v>7740</v>
       </c>
       <c r="B188" t="s">
-        <v>397</v>
+        <v>382</v>
       </c>
       <c r="C188" t="s">
-        <v>522</v>
+        <v>507</v>
       </c>
       <c r="D188">
         <v>3</v>
@@ -7912,10 +7867,10 @@
         <v>7735</v>
       </c>
       <c r="B189" t="s">
-        <v>438</v>
+        <v>423</v>
       </c>
       <c r="C189" t="s">
-        <v>439</v>
+        <v>424</v>
       </c>
       <c r="D189">
         <v>3</v>
@@ -7942,10 +7897,10 @@
         <v>7736</v>
       </c>
       <c r="B190" t="s">
-        <v>442</v>
+        <v>427</v>
       </c>
       <c r="C190" t="s">
-        <v>443</v>
+        <v>428</v>
       </c>
       <c r="D190">
         <v>3</v>
@@ -7972,10 +7927,10 @@
         <v>7737</v>
       </c>
       <c r="B191" t="s">
-        <v>389</v>
+        <v>374</v>
       </c>
       <c r="C191" t="s">
-        <v>523</v>
+        <v>508</v>
       </c>
       <c r="D191">
         <v>3</v>
@@ -8002,10 +7957,10 @@
         <v>7738</v>
       </c>
       <c r="B192" t="s">
-        <v>391</v>
+        <v>376</v>
       </c>
       <c r="C192" t="s">
-        <v>524</v>
+        <v>509</v>
       </c>
       <c r="D192">
         <v>3</v>
@@ -8032,10 +7987,10 @@
         <v>7739</v>
       </c>
       <c r="B193" t="s">
-        <v>525</v>
+        <v>510</v>
       </c>
       <c r="C193" t="s">
-        <v>526</v>
+        <v>511</v>
       </c>
       <c r="D193">
         <v>3</v>
@@ -8062,10 +8017,10 @@
         <v>7734</v>
       </c>
       <c r="B194" t="s">
-        <v>446</v>
+        <v>431</v>
       </c>
       <c r="C194" t="s">
-        <v>527</v>
+        <v>512</v>
       </c>
       <c r="D194">
         <v>3</v>
@@ -8092,10 +8047,10 @@
         <v>7741</v>
       </c>
       <c r="B195" t="s">
-        <v>393</v>
+        <v>378</v>
       </c>
       <c r="C195" t="s">
-        <v>528</v>
+        <v>513</v>
       </c>
       <c r="D195">
         <v>3</v>
@@ -8122,10 +8077,10 @@
         <v>7742</v>
       </c>
       <c r="B196" t="s">
-        <v>529</v>
+        <v>514</v>
       </c>
       <c r="C196" t="s">
-        <v>530</v>
+        <v>515</v>
       </c>
       <c r="D196">
         <v>3</v>
@@ -8152,10 +8107,10 @@
         <v>7743</v>
       </c>
       <c r="B197" t="s">
-        <v>448</v>
+        <v>433</v>
       </c>
       <c r="C197" t="s">
-        <v>531</v>
+        <v>516</v>
       </c>
       <c r="D197">
         <v>3</v>
@@ -8182,10 +8137,10 @@
         <v>7749</v>
       </c>
       <c r="B198" t="s">
-        <v>452</v>
+        <v>437</v>
       </c>
       <c r="C198" t="s">
-        <v>532</v>
+        <v>517</v>
       </c>
       <c r="D198">
         <v>4</v>
@@ -8212,10 +8167,10 @@
         <v>7745</v>
       </c>
       <c r="B199" t="s">
-        <v>456</v>
+        <v>441</v>
       </c>
       <c r="C199" t="s">
-        <v>533</v>
+        <v>518</v>
       </c>
       <c r="D199">
         <v>4</v>
@@ -8242,10 +8197,10 @@
         <v>7746</v>
       </c>
       <c r="B200" t="s">
-        <v>403</v>
+        <v>388</v>
       </c>
       <c r="C200" t="s">
-        <v>534</v>
+        <v>519</v>
       </c>
       <c r="D200">
         <v>4</v>
@@ -8272,10 +8227,10 @@
         <v>7747</v>
       </c>
       <c r="B201" t="s">
-        <v>440</v>
+        <v>425</v>
       </c>
       <c r="C201" t="s">
-        <v>535</v>
+        <v>520</v>
       </c>
       <c r="D201">
         <v>4</v>
@@ -8302,10 +8257,10 @@
         <v>7748</v>
       </c>
       <c r="B202" t="s">
-        <v>395</v>
+        <v>380</v>
       </c>
       <c r="C202" t="s">
-        <v>536</v>
+        <v>521</v>
       </c>
       <c r="D202">
         <v>4</v>
@@ -8332,10 +8287,10 @@
         <v>7744</v>
       </c>
       <c r="B203" t="s">
-        <v>399</v>
+        <v>384</v>
       </c>
       <c r="C203" t="s">
-        <v>537</v>
+        <v>522</v>
       </c>
       <c r="D203">
         <v>4</v>
@@ -8362,10 +8317,10 @@
         <v>7750</v>
       </c>
       <c r="B204" t="s">
-        <v>405</v>
+        <v>390</v>
       </c>
       <c r="C204" t="s">
-        <v>538</v>
+        <v>523</v>
       </c>
       <c r="D204">
         <v>4</v>
@@ -8392,10 +8347,10 @@
         <v>7751</v>
       </c>
       <c r="B205" t="s">
-        <v>454</v>
+        <v>439</v>
       </c>
       <c r="C205" t="s">
-        <v>455</v>
+        <v>440</v>
       </c>
       <c r="D205">
         <v>4</v>
@@ -8422,10 +8377,10 @@
         <v>7752</v>
       </c>
       <c r="B206" t="s">
-        <v>409</v>
+        <v>394</v>
       </c>
       <c r="C206" t="s">
-        <v>539</v>
+        <v>524</v>
       </c>
       <c r="D206">
         <v>4</v>
@@ -8452,10 +8407,10 @@
         <v>7753</v>
       </c>
       <c r="B207" t="s">
-        <v>450</v>
+        <v>435</v>
       </c>
       <c r="C207" t="s">
-        <v>451</v>
+        <v>436</v>
       </c>
       <c r="D207">
         <v>4</v>
@@ -8482,10 +8437,10 @@
         <v>7763</v>
       </c>
       <c r="B208" t="s">
-        <v>444</v>
+        <v>429</v>
       </c>
       <c r="C208" t="s">
-        <v>540</v>
+        <v>525</v>
       </c>
       <c r="D208">
         <v>4</v>
@@ -8512,10 +8467,10 @@
         <v>7754</v>
       </c>
       <c r="B209" t="s">
-        <v>411</v>
+        <v>396</v>
       </c>
       <c r="C209" t="s">
-        <v>541</v>
+        <v>526</v>
       </c>
       <c r="D209">
         <v>5</v>
@@ -8542,10 +8497,10 @@
         <v>7755</v>
       </c>
       <c r="B210" t="s">
-        <v>427</v>
+        <v>412</v>
       </c>
       <c r="C210" t="s">
-        <v>542</v>
+        <v>527</v>
       </c>
       <c r="D210">
         <v>5</v>
@@ -8572,10 +8527,10 @@
         <v>7756</v>
       </c>
       <c r="B211" t="s">
-        <v>458</v>
+        <v>443</v>
       </c>
       <c r="C211" t="s">
-        <v>459</v>
+        <v>444</v>
       </c>
       <c r="D211">
         <v>5</v>
@@ -8602,10 +8557,10 @@
         <v>7757</v>
       </c>
       <c r="B212" t="s">
-        <v>460</v>
+        <v>445</v>
       </c>
       <c r="C212" t="s">
-        <v>543</v>
+        <v>528</v>
       </c>
       <c r="D212">
         <v>5</v>
@@ -8632,10 +8587,10 @@
         <v>7758</v>
       </c>
       <c r="B213" t="s">
-        <v>429</v>
+        <v>414</v>
       </c>
       <c r="C213" t="s">
-        <v>430</v>
+        <v>415</v>
       </c>
       <c r="D213">
         <v>5</v>
@@ -8662,10 +8617,10 @@
         <v>7760</v>
       </c>
       <c r="B214" t="s">
-        <v>544</v>
+        <v>529</v>
       </c>
       <c r="C214" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="D214">
         <v>5</v>
@@ -8681,7 +8636,7 @@
         <v>254</v>
       </c>
       <c r="H214" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I214">
         <v>2</v>
@@ -14216,8 +14171,8 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>114</v>
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -14226,21 +14181,21 @@
         <v>46038</v>
       </c>
       <c r="D2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F2" t="s">
         <v>115</v>
       </c>
-      <c r="E2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>116</v>
       </c>
-      <c r="G2" t="s">
-        <v>117</v>
-      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>118</v>
+      <c r="A3">
+        <v>2</v>
       </c>
       <c r="B3">
         <v>23</v>
@@ -14249,21 +14204,21 @@
         <v>46044</v>
       </c>
       <c r="D3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>121</v>
+      <c r="A4">
+        <v>3</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -14272,21 +14227,21 @@
         <v>46049</v>
       </c>
       <c r="D4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F4" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G4" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>125</v>
+      <c r="A5">
+        <v>4</v>
       </c>
       <c r="B5">
         <v>12</v>
@@ -14295,21 +14250,21 @@
         <v>46045</v>
       </c>
       <c r="D5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>129</v>
+      <c r="A6">
+        <v>5</v>
       </c>
       <c r="B6">
         <v>47</v>
@@ -14318,21 +14273,21 @@
         <v>46051</v>
       </c>
       <c r="D6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F6" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="G6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>131</v>
+      <c r="A7">
+        <v>6</v>
       </c>
       <c r="B7">
         <v>12</v>
@@ -14341,21 +14296,21 @@
         <v>46049</v>
       </c>
       <c r="D7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G7" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>133</v>
+      <c r="A8">
+        <v>7</v>
       </c>
       <c r="B8">
         <v>23</v>
@@ -14364,21 +14319,21 @@
         <v>46056</v>
       </c>
       <c r="D8" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G8" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>134</v>
+      <c r="A9">
+        <v>8</v>
       </c>
       <c r="B9">
         <v>23</v>
@@ -14387,21 +14342,21 @@
         <v>46063</v>
       </c>
       <c r="D9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F9" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G9" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>135</v>
+      <c r="A10">
+        <v>9</v>
       </c>
       <c r="B10">
         <v>23</v>
@@ -14410,21 +14365,21 @@
         <v>46070</v>
       </c>
       <c r="D10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F10" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G10" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>136</v>
+      <c r="A11">
+        <v>10</v>
       </c>
       <c r="B11">
         <v>12</v>
@@ -14433,21 +14388,21 @@
         <v>46056</v>
       </c>
       <c r="D11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F11" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="G11" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>139</v>
+      <c r="A12">
+        <v>11</v>
       </c>
       <c r="B12">
         <v>12</v>
@@ -14456,21 +14411,21 @@
         <v>46063</v>
       </c>
       <c r="D12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F12" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="G12" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>140</v>
+      <c r="A13">
+        <v>12</v>
       </c>
       <c r="B13">
         <v>12</v>
@@ -14479,21 +14434,21 @@
         <v>46070</v>
       </c>
       <c r="D13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F13" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="G13" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>141</v>
+      <c r="A14">
+        <v>13</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -14502,21 +14457,21 @@
         <v>46058</v>
       </c>
       <c r="D14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F14" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="G14" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>144</v>
+      <c r="A15">
+        <v>14</v>
       </c>
       <c r="B15">
         <v>23</v>
@@ -14525,21 +14480,21 @@
         <v>46059</v>
       </c>
       <c r="D15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F15" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="G15" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>147</v>
+      <c r="A16">
+        <v>15</v>
       </c>
       <c r="B16">
         <v>12</v>
@@ -14548,16 +14503,16 @@
         <v>46112</v>
       </c>
       <c r="D16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F16" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="G16" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -14580,10 +14535,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>54</v>
@@ -14595,7 +14550,7 @@
         <v>50</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -14610,57 +14565,57 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>114</v>
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="C2" t="s">
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="E2" s="3">
         <v>46038.654861111107</v>
@@ -14688,17 +14643,17 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>118</v>
+      <c r="A3">
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="C3" t="s">
         <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="E3" s="3">
         <v>46044.75</v>
@@ -14726,17 +14681,17 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>121</v>
+      <c r="A4">
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="C4" t="s">
         <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="E4" s="3">
         <v>46049.416666666657</v>
@@ -14764,17 +14719,17 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>125</v>
+      <c r="A5">
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="C5" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="D5" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="E5" s="3">
         <v>46045.375</v>
@@ -14802,17 +14757,17 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>129</v>
+      <c r="A6">
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="C6" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="D6" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="E6" s="3">
         <v>46051.666666666657</v>
@@ -14840,17 +14795,17 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>131</v>
+      <c r="A7">
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="C7" t="s">
         <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="E7" s="3">
         <v>46049.416666666657</v>
@@ -14878,17 +14833,17 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>133</v>
+      <c r="A8">
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="C8" t="s">
         <v>32</v>
       </c>
       <c r="D8" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="E8" s="3">
         <v>46056.416666666657</v>
@@ -14916,17 +14871,17 @@
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>134</v>
+      <c r="A9">
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="C9" t="s">
         <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="E9" s="3">
         <v>46063.416666666657</v>
@@ -14954,17 +14909,17 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>135</v>
+      <c r="A10">
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="C10" t="s">
         <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="E10" s="3">
         <v>46070.416666666657</v>
@@ -14992,17 +14947,17 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>136</v>
+      <c r="A11">
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C11" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="D11" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="E11" s="3">
         <v>46056.6875</v>
@@ -15030,17 +14985,17 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>139</v>
+      <c r="A12">
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C12" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="D12" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="E12" s="3">
         <v>46063.6875</v>
@@ -15068,17 +15023,17 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>140</v>
+      <c r="A13">
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C13" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="D13" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="E13" s="3">
         <v>46070.6875</v>
@@ -15106,17 +15061,17 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>141</v>
+      <c r="A14">
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C14" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="D14" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="E14" s="3">
         <v>46058.479166666657</v>
@@ -15144,17 +15099,17 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>144</v>
+      <c r="A15">
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="C15" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="D15" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="E15" s="3">
         <v>46059.727777777778</v>
@@ -15182,17 +15137,17 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>147</v>
+      <c r="A16">
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="C16" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="D16" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="E16" s="3">
         <v>46112.625</v>
@@ -15248,49 +15203,49 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="B2" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="C2" t="s">
-        <v>184</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="B3" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
       <c r="C3" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="B4" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="C4" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
       <c r="D4" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="B5" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="C5" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -15312,49 +15267,49 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="B7" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="C7" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="D7" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="B8" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="C8" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="B9" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="C9" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="B10" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="C10" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -15369,13 +15324,13 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>49</v>
@@ -15595,34 +15550,34 @@
         <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -15691,7 +15646,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="C2" t="s">
         <v>31</v>
@@ -15715,7 +15670,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="s">
-        <v>545</v>
+        <v>530</v>
       </c>
       <c r="O2" t="s">
         <v>35</v>
@@ -15726,7 +15681,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>576</v>
+        <v>561</v>
       </c>
       <c r="C3" t="s">
         <v>31</v>
@@ -15753,7 +15708,7 @@
         <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>546</v>
+        <v>531</v>
       </c>
       <c r="O3" t="s">
         <v>35</v>
@@ -15764,7 +15719,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>575</v>
+        <v>560</v>
       </c>
       <c r="C4" t="s">
         <v>31</v>
@@ -15791,7 +15746,7 @@
         <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>547</v>
+        <v>532</v>
       </c>
       <c r="O4" t="s">
         <v>35</v>
@@ -15802,7 +15757,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>577</v>
+        <v>562</v>
       </c>
       <c r="C5" t="s">
         <v>31</v>
@@ -15826,7 +15781,7 @@
         <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>548</v>
+        <v>533</v>
       </c>
       <c r="O5" t="s">
         <v>35</v>
@@ -15837,7 +15792,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="C6" t="s">
         <v>31</v>
@@ -15875,7 +15830,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C7" t="s">
         <v>31</v>
@@ -15902,7 +15857,7 @@
         <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>547</v>
+        <v>532</v>
       </c>
       <c r="O7" t="s">
         <v>35</v>
@@ -15913,7 +15868,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="C8" t="s">
         <v>31</v>
@@ -15940,7 +15895,7 @@
         <v>1</v>
       </c>
       <c r="K8" t="s">
-        <v>549</v>
+        <v>534</v>
       </c>
       <c r="O8" t="s">
         <v>35</v>
@@ -15951,7 +15906,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>578</v>
+        <v>563</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -15978,7 +15933,7 @@
         <v>1</v>
       </c>
       <c r="K9" t="s">
-        <v>550</v>
+        <v>535</v>
       </c>
       <c r="O9" t="s">
         <v>35</v>
@@ -15989,7 +15944,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>579</v>
+        <v>564</v>
       </c>
       <c r="C10" t="s">
         <v>31</v>
@@ -16016,7 +15971,7 @@
         <v>1</v>
       </c>
       <c r="K10" t="s">
-        <v>551</v>
+        <v>536</v>
       </c>
       <c r="O10" t="s">
         <v>35</v>
@@ -16027,7 +15982,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>580</v>
+        <v>565</v>
       </c>
       <c r="C11" t="s">
         <v>31</v>
@@ -16054,7 +16009,7 @@
         <v>1</v>
       </c>
       <c r="K11" t="s">
-        <v>552</v>
+        <v>537</v>
       </c>
       <c r="O11" t="s">
         <v>35</v>
@@ -16065,7 +16020,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="C12" t="s">
         <v>31</v>
@@ -16092,10 +16047,10 @@
         <v>1</v>
       </c>
       <c r="K12" t="s">
-        <v>553</v>
+        <v>538</v>
       </c>
       <c r="L12" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="O12" t="s">
         <v>35</v>
@@ -16133,10 +16088,10 @@
         <v>1</v>
       </c>
       <c r="K13" t="s">
-        <v>554</v>
+        <v>539</v>
       </c>
       <c r="L13" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="O13" t="s">
         <v>35</v>
@@ -16147,7 +16102,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="C14" t="s">
         <v>31</v>
@@ -16171,10 +16126,10 @@
         <v>1</v>
       </c>
       <c r="K14" t="s">
-        <v>555</v>
+        <v>540</v>
       </c>
       <c r="L14" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="O14" t="s">
         <v>35</v>
@@ -16185,7 +16140,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="C15" t="s">
         <v>31</v>
@@ -16209,10 +16164,10 @@
         <v>1</v>
       </c>
       <c r="K15" t="s">
-        <v>556</v>
+        <v>541</v>
       </c>
       <c r="L15" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="O15" t="s">
         <v>35</v>
@@ -16223,7 +16178,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>221</v>
+        <v>206</v>
       </c>
       <c r="C16" t="s">
         <v>31</v>
@@ -16232,7 +16187,7 @@
         <v>4</v>
       </c>
       <c r="K16" t="s">
-        <v>557</v>
+        <v>542</v>
       </c>
       <c r="O16" t="s">
         <v>35</v>
@@ -16243,7 +16198,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>222</v>
+        <v>207</v>
       </c>
       <c r="C17" t="s">
         <v>37</v>
@@ -16270,7 +16225,7 @@
         <v>1</v>
       </c>
       <c r="K17" t="s">
-        <v>558</v>
+        <v>543</v>
       </c>
       <c r="O17" t="s">
         <v>35</v>
@@ -16281,7 +16236,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>223</v>
+        <v>208</v>
       </c>
       <c r="C18" t="s">
         <v>37</v>
@@ -16308,7 +16263,7 @@
         <v>1</v>
       </c>
       <c r="K18" t="s">
-        <v>559</v>
+        <v>544</v>
       </c>
       <c r="O18" t="s">
         <v>35</v>
@@ -16319,7 +16274,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="C19" t="s">
         <v>37</v>
@@ -16346,7 +16301,7 @@
         <v>1</v>
       </c>
       <c r="K19" t="s">
-        <v>560</v>
+        <v>545</v>
       </c>
       <c r="O19" t="s">
         <v>35</v>
@@ -16357,7 +16312,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="C20" t="s">
         <v>37</v>
@@ -16384,7 +16339,7 @@
         <v>1</v>
       </c>
       <c r="K20" t="s">
-        <v>561</v>
+        <v>546</v>
       </c>
       <c r="O20" t="s">
         <v>35</v>
@@ -16395,7 +16350,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="C21" t="s">
         <v>37</v>
@@ -16422,7 +16377,7 @@
         <v>1</v>
       </c>
       <c r="K21" t="s">
-        <v>562</v>
+        <v>547</v>
       </c>
       <c r="O21" t="s">
         <v>35</v>
@@ -16433,7 +16388,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="C22" t="s">
         <v>37</v>
@@ -16460,7 +16415,7 @@
         <v>1</v>
       </c>
       <c r="K22" t="s">
-        <v>563</v>
+        <v>548</v>
       </c>
       <c r="O22" t="s">
         <v>35</v>
@@ -16471,7 +16426,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C23" t="s">
         <v>37</v>
@@ -16498,7 +16453,7 @@
         <v>1</v>
       </c>
       <c r="K23" t="s">
-        <v>564</v>
+        <v>549</v>
       </c>
       <c r="O23" t="s">
         <v>35</v>
@@ -16536,7 +16491,7 @@
         <v>1</v>
       </c>
       <c r="K24" t="s">
-        <v>565</v>
+        <v>550</v>
       </c>
       <c r="O24" t="s">
         <v>35</v>
@@ -16547,7 +16502,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="C25" t="s">
         <v>37</v>
@@ -16574,7 +16529,7 @@
         <v>1</v>
       </c>
       <c r="K25" t="s">
-        <v>566</v>
+        <v>551</v>
       </c>
       <c r="O25" t="s">
         <v>35</v>
@@ -16585,7 +16540,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="C26" t="s">
         <v>37</v>
@@ -16609,10 +16564,10 @@
         <v>1</v>
       </c>
       <c r="K26" t="s">
-        <v>567</v>
+        <v>552</v>
       </c>
       <c r="L26" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="O26" t="s">
         <v>35</v>
@@ -16623,7 +16578,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>232</v>
+        <v>217</v>
       </c>
       <c r="C27" t="s">
         <v>37</v>
@@ -16644,7 +16599,7 @@
         <v>0</v>
       </c>
       <c r="K27" t="s">
-        <v>568</v>
+        <v>553</v>
       </c>
       <c r="O27" t="s">
         <v>35</v>
@@ -16655,7 +16610,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="C28" t="s">
         <v>37</v>
@@ -16679,7 +16634,7 @@
         <v>0</v>
       </c>
       <c r="K28" t="s">
-        <v>569</v>
+        <v>554</v>
       </c>
       <c r="O28" t="s">
         <v>35</v>
@@ -16690,7 +16645,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
       <c r="C29" t="s">
         <v>37</v>
@@ -16714,7 +16669,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="O29" t="s">
         <v>35</v>
@@ -16725,7 +16680,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>235</v>
+        <v>220</v>
       </c>
       <c r="C30" t="s">
         <v>37</v>
@@ -16754,7 +16709,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>236</v>
+        <v>221</v>
       </c>
       <c r="C31" t="s">
         <v>31</v>
@@ -16766,7 +16721,7 @@
         <v>442</v>
       </c>
       <c r="L31" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
       <c r="O31" t="s">
         <v>35</v>
@@ -16777,7 +16732,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="C32" t="s">
         <v>31</v>
@@ -16794,7 +16749,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="C33" t="s">
         <v>42</v>
@@ -16809,7 +16764,7 @@
         <v>1</v>
       </c>
       <c r="K33" t="s">
-        <v>571</v>
+        <v>556</v>
       </c>
       <c r="O33" t="s">
         <v>35</v>
@@ -16820,7 +16775,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>269</v>
+        <v>254</v>
       </c>
       <c r="C34" t="s">
         <v>42</v>
@@ -16844,7 +16799,7 @@
         <v>0</v>
       </c>
       <c r="K34" t="s">
-        <v>572</v>
+        <v>557</v>
       </c>
       <c r="O34" t="s">
         <v>35</v>
@@ -16855,7 +16810,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>239</v>
+        <v>224</v>
       </c>
       <c r="C35" t="s">
         <v>42</v>
@@ -16867,7 +16822,7 @@
         <v>30</v>
       </c>
       <c r="K35" t="s">
-        <v>573</v>
+        <v>558</v>
       </c>
       <c r="O35" t="s">
         <v>35</v>
@@ -16878,7 +16833,7 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>240</v>
+        <v>225</v>
       </c>
       <c r="C36" t="s">
         <v>42</v>
@@ -16902,7 +16857,7 @@
         <v>0</v>
       </c>
       <c r="K36" t="s">
-        <v>574</v>
+        <v>559</v>
       </c>
       <c r="O36" t="s">
         <v>35</v>
@@ -16913,7 +16868,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="C37" t="s">
         <v>42</v>
@@ -16937,7 +16892,7 @@
         <v>149</v>
       </c>
       <c r="L37" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="O37" t="s">
         <v>35</v>
@@ -16948,7 +16903,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>243</v>
+        <v>228</v>
       </c>
       <c r="C38" t="s">
         <v>42</v>
@@ -16963,7 +16918,7 @@
         <v>1</v>
       </c>
       <c r="L38" t="s">
-        <v>244</v>
+        <v>229</v>
       </c>
       <c r="O38" t="s">
         <v>35</v>
@@ -16974,7 +16929,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="C39" t="s">
         <v>42</v>
@@ -16998,7 +16953,7 @@
         <v>1</v>
       </c>
       <c r="L39" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="O39" t="s">
         <v>35</v>
@@ -17009,7 +16964,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="C40" t="s">
         <v>42</v>
@@ -17029,7 +16984,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="O41" t="s">
         <v>35</v>
@@ -17040,7 +16995,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="O42" t="s">
         <v>35</v>
@@ -17051,7 +17006,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
       <c r="O43" t="s">
         <v>35</v>
@@ -17062,7 +17017,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="O44" t="s">
         <v>35</v>
@@ -17073,7 +17028,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>252</v>
+        <v>237</v>
       </c>
       <c r="O45" t="s">
         <v>35</v>
@@ -17084,7 +17039,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>253</v>
+        <v>238</v>
       </c>
       <c r="O46" t="s">
         <v>35</v>
@@ -17095,7 +17050,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>254</v>
+        <v>239</v>
       </c>
       <c r="O47" t="s">
         <v>35</v>
@@ -17106,7 +17061,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>255</v>
+        <v>240</v>
       </c>
       <c r="O48" t="s">
         <v>35</v>
@@ -17117,7 +17072,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>256</v>
+        <v>241</v>
       </c>
       <c r="O49" t="s">
         <v>35</v>
@@ -17128,7 +17083,7 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>257</v>
+        <v>242</v>
       </c>
       <c r="O50" t="s">
         <v>35</v>
@@ -17139,7 +17094,7 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>258</v>
+        <v>243</v>
       </c>
       <c r="O51" t="s">
         <v>35</v>
@@ -17150,7 +17105,7 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="O52" t="s">
         <v>35</v>
@@ -17161,7 +17116,7 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="O53" t="s">
         <v>35</v>
@@ -17172,7 +17127,7 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>261</v>
+        <v>246</v>
       </c>
       <c r="O54" t="s">
         <v>35</v>
@@ -17183,7 +17138,7 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>262</v>
+        <v>247</v>
       </c>
       <c r="O55" t="s">
         <v>35</v>
@@ -17194,7 +17149,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="O56" t="s">
         <v>35</v>
@@ -17205,7 +17160,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>264</v>
+        <v>249</v>
       </c>
       <c r="O57" t="s">
         <v>35</v>
@@ -17216,7 +17171,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>265</v>
+        <v>250</v>
       </c>
       <c r="O58" t="s">
         <v>35</v>
@@ -17227,7 +17182,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>266</v>
+        <v>251</v>
       </c>
       <c r="O59" t="s">
         <v>35</v>
@@ -17238,7 +17193,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>267</v>
+        <v>252</v>
       </c>
       <c r="O60" t="s">
         <v>35</v>
@@ -17249,7 +17204,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>581</v>
+        <v>566</v>
       </c>
       <c r="O61" t="s">
         <v>35</v>

</xml_diff>